<commit_message>
Deploying to gh-pages from @ koodiklinikka/palkkakysely@1d14bfe765e80530437cee730768a5225480e314 🚀
</commit_message>
<xml_diff>
--- a/2024/raw-en.xlsx
+++ b/2024/raw-en.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Form responses 1" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Form responses 1" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Form responses 1'!$A$1:$Z$53</definedName>
@@ -651,223 +651,42 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="1">
     <border/>
-    <border>
-      <left style="thin">
-        <color rgb="FF442F65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF5B3F86"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF442F65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF442F65"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF5B3F86"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF5B3F86"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF442F65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF442F65"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF5B3F86"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF442F65"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF442F65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF442F65"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF442F65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFFFFFFF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFFFFFFF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFFFFFFF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFFFFFFF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF442F65"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF442F65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF8F9FA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFF8F9FA"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFF8F9FA"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF8F9FA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFF8F9FA"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFF8F9FA"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF442F65"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF8F9FA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFF8F9FA"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF442F65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF8F9FA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF442F65"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFF8F9FA"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF8F9FA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF442F65"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <font/>
       <fill>
@@ -905,12 +724,29 @@
       </fill>
       <border/>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF5B3F86"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF5B3F86"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF5B3F86"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF5B3F86"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="3" pivot="0" name="Form responses 1-style">
+    <tableStyle count="4" pivot="0" name="Form responses 1-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
   </tableStyles>
 </styleSheet>
@@ -918,6 +754,10 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1184,2728 +1024,2728 @@
     <col customWidth="1" min="27" max="32" width="18.88"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4">
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="2">
         <v>45572.52955902778</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="B2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="3">
         <v>16.0</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="3">
         <v>0.0</v>
       </c>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="5" t="s">
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="Q2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="R2" s="5">
-        <v>100.0</v>
-      </c>
-      <c r="S2" s="5">
+      <c r="R2" s="3">
+        <v>100.0</v>
+      </c>
+      <c r="S2" s="3">
         <v>0.0</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="U2" s="5">
+      <c r="U2" s="3">
         <v>8400.0</v>
       </c>
-      <c r="V2" s="5">
+      <c r="V2" s="3">
         <v>0.0</v>
       </c>
-      <c r="W2" s="5" t="s">
+      <c r="W2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="X2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y2" s="6"/>
-      <c r="Z2" s="7"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="8">
+      <c r="X2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="5">
         <v>45572.53306934028</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="6">
         <v>8.0</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="6">
         <v>2.0</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="R3" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S3" s="9">
+      <c r="R3" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S3" s="6">
         <v>70.0</v>
       </c>
-      <c r="T3" s="9" t="s">
+      <c r="T3" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="U3" s="9">
+      <c r="U3" s="6">
         <v>5300.0</v>
       </c>
-      <c r="V3" s="9">
+      <c r="V3" s="6">
         <v>75000.0</v>
       </c>
-      <c r="X3" s="9" t="s">
+      <c r="X3" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="10">
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="5">
         <v>45572.88351467592</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="6">
         <v>7.0</v>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="6">
         <v>70.0</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="M4" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="N4" s="11" t="s">
+      <c r="N4" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="8">
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="5">
         <v>45575.75525584491</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="C5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="6">
         <v>10.0</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="6">
         <v>-6.0</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="6">
         <v>3.0</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="6">
         <v>90.0</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="6">
         <v>109000.0</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="M5" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="N5" s="9" t="s">
+      <c r="N5" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="10">
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="5">
         <v>45576.52333413194</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="11" t="s">
+      <c r="C6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="6">
         <v>25.0</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="6">
         <v>0.0</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="6">
         <v>13.0</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="6">
         <v>95.0</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="6">
         <v>165000.0</v>
       </c>
-      <c r="M6" s="11" t="s">
+      <c r="M6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="N6" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8">
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="5">
         <v>45576.5281666088</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="B7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="6">
         <v>9.0</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="6">
         <v>4.0</v>
       </c>
-      <c r="P7" s="9" t="s">
+      <c r="P7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q7" s="9" t="s">
+      <c r="Q7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R7" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S7" s="9">
+      <c r="R7" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S7" s="6">
         <v>10.0</v>
       </c>
-      <c r="U7" s="9">
+      <c r="U7" s="6">
         <v>5080.0</v>
       </c>
-      <c r="V7" s="9">
+      <c r="V7" s="6">
         <v>62000.0</v>
       </c>
-      <c r="X7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="12" t="s">
+      <c r="X7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10">
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="5">
         <v>45576.528633124995</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="11" t="s">
+      <c r="B8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="6">
         <v>11.0</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="P8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q8" s="11" t="s">
+      <c r="Q8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R8" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S8" s="11">
+      <c r="R8" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S8" s="6">
         <v>0.0</v>
       </c>
-      <c r="T8" s="11" t="s">
+      <c r="T8" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="U8" s="11">
+      <c r="U8" s="6">
         <v>6000.0</v>
       </c>
-      <c r="V8" s="11">
+      <c r="V8" s="6">
         <v>72000.0</v>
       </c>
-      <c r="X8" s="11" t="s">
+      <c r="X8" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8">
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="5">
         <v>45576.53063306713</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="6">
         <v>23.0</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="6">
         <v>0.0</v>
       </c>
-      <c r="P9" s="9" t="s">
+      <c r="P9" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q9" s="9" t="s">
+      <c r="Q9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R9" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S9" s="9">
+      <c r="R9" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S9" s="6">
         <v>95.0</v>
       </c>
-      <c r="T9" s="9" t="s">
+      <c r="T9" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="U9" s="9">
+      <c r="U9" s="6">
         <v>6400.0</v>
       </c>
-      <c r="V9" s="9">
+      <c r="V9" s="6">
         <v>76800.0</v>
       </c>
-      <c r="X9" s="9" t="s">
+      <c r="X9" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="10">
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="5">
         <v>45576.53280670139</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="11" t="s">
+      <c r="C10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="6">
         <v>6.0</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="6">
         <v>0.0</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="6">
         <v>2.0</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="K10" s="11">
+      <c r="K10" s="6">
         <v>92.0</v>
       </c>
-      <c r="L10" s="11">
+      <c r="L10" s="6">
         <v>86000.0</v>
       </c>
-      <c r="M10" s="11" t="s">
+      <c r="M10" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="Z10" s="13" t="s">
+      <c r="Z10" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8">
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="5">
         <v>45576.533064247684</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="B11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="6">
         <v>7.0</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="6">
         <v>15.0</v>
       </c>
-      <c r="O11" s="9" t="s">
+      <c r="O11" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="P11" s="9" t="s">
+      <c r="P11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q11" s="9" t="s">
+      <c r="Q11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R11" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S11" s="9">
+      <c r="R11" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S11" s="6">
         <v>80.0</v>
       </c>
-      <c r="T11" s="9" t="s">
+      <c r="T11" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="U11" s="9">
+      <c r="U11" s="6">
         <v>6100.0</v>
       </c>
-      <c r="V11" s="9">
+      <c r="V11" s="6">
         <v>100000.0</v>
       </c>
-      <c r="W11" s="9" t="s">
+      <c r="W11" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="X11" s="9" t="s">
+      <c r="X11" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="Z11" s="12" t="s">
+      <c r="Z11" s="6" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10">
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="A12" s="5">
         <v>45576.53863144676</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="11" t="s">
+      <c r="B12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="6">
         <v>3.0</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="6">
         <v>5.0</v>
       </c>
-      <c r="O12" s="11" t="s">
+      <c r="O12" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="P12" s="11" t="s">
+      <c r="P12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q12" s="11" t="s">
+      <c r="Q12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R12" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S12" s="11">
+      <c r="R12" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S12" s="6">
         <v>10.0</v>
       </c>
-      <c r="T12" s="11" t="s">
+      <c r="T12" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="U12" s="11">
+      <c r="U12" s="6">
         <v>4000.0</v>
       </c>
-      <c r="V12" s="11">
+      <c r="V12" s="6">
         <v>52000.0</v>
       </c>
-      <c r="X12" s="11" t="s">
+      <c r="X12" s="6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8">
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="5">
         <v>45576.54224546296</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="6">
         <v>4.0</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="6">
         <v>20.0</v>
       </c>
-      <c r="P13" s="9" t="s">
+      <c r="P13" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q13" s="9" t="s">
+      <c r="Q13" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R13" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S13" s="9">
+      <c r="R13" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S13" s="6">
         <v>80.0</v>
       </c>
-      <c r="T13" s="9" t="s">
+      <c r="T13" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="U13" s="9">
+      <c r="U13" s="6">
         <v>5500.0</v>
       </c>
-      <c r="V13" s="9">
+      <c r="V13" s="6">
         <v>70.0</v>
       </c>
-      <c r="X13" s="9" t="s">
+      <c r="X13" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10">
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="5">
         <v>45576.547714953704</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="11" t="s">
+      <c r="B14" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="6">
         <v>15.0</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="6">
         <v>20.0</v>
       </c>
-      <c r="P14" s="11" t="s">
+      <c r="P14" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q14" s="11" t="s">
+      <c r="Q14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R14" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S14" s="11">
+      <c r="R14" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S14" s="6">
         <v>2.0</v>
       </c>
-      <c r="T14" s="11" t="s">
+      <c r="T14" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="U14" s="11">
+      <c r="U14" s="6">
         <v>6500.0</v>
       </c>
-      <c r="V14" s="11">
+      <c r="V14" s="6">
         <v>78000.0</v>
       </c>
-      <c r="X14" s="11" t="s">
+      <c r="X14" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8">
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="5">
         <v>45576.556192118056</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="9" t="s">
+      <c r="B15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="6">
         <v>8.0</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="O15" s="9" t="s">
+      <c r="O15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P15" s="9" t="s">
+      <c r="P15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q15" s="9" t="s">
+      <c r="Q15" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R15" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S15" s="9">
+      <c r="R15" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S15" s="6">
         <v>20.0</v>
       </c>
-      <c r="T15" s="9" t="s">
+      <c r="T15" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="U15" s="9">
+      <c r="U15" s="6">
         <v>5074.0</v>
       </c>
-      <c r="V15" s="9">
+      <c r="V15" s="6">
         <v>60888.0</v>
       </c>
-      <c r="X15" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10">
+      <c r="X15" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="5">
         <v>45576.56048519676</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="B16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="6">
         <v>2.5</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="6">
         <v>2.5</v>
       </c>
-      <c r="O16" s="11" t="s">
+      <c r="O16" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="P16" s="11" t="s">
+      <c r="P16" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="Q16" s="11" t="s">
+      <c r="Q16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R16" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S16" s="11">
+      <c r="R16" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S16" s="6">
         <v>0.0</v>
       </c>
-      <c r="T16" s="11" t="s">
+      <c r="T16" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="U16" s="11">
+      <c r="U16" s="6">
         <v>3200.0</v>
       </c>
-      <c r="V16" s="11">
+      <c r="V16" s="6">
         <v>38400.0</v>
       </c>
-      <c r="X16" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8">
+      <c r="X16" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="5">
         <v>45576.56309826389</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="B17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="6">
         <v>17.0</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="6">
         <v>2.0</v>
       </c>
-      <c r="O17" s="14" t="s">
+      <c r="O17" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="P17" s="9" t="s">
+      <c r="P17" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q17" s="9" t="s">
+      <c r="Q17" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R17" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S17" s="9">
+      <c r="R17" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S17" s="6">
         <v>40.0</v>
       </c>
-      <c r="T17" s="9" t="s">
+      <c r="T17" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="U17" s="9">
+      <c r="U17" s="6">
         <v>6630.0</v>
       </c>
-      <c r="V17" s="9">
+      <c r="V17" s="6">
         <v>93000.0</v>
       </c>
-      <c r="W17" s="9" t="s">
+      <c r="W17" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="X17" s="9" t="s">
+      <c r="X17" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="10">
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="5">
         <v>45576.602097361116</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D18" s="11" t="s">
+      <c r="B18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="6">
         <v>11.0</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="H18" s="11">
+      <c r="H18" s="6">
         <v>0.0</v>
       </c>
-      <c r="P18" s="11" t="s">
+      <c r="P18" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="Q18" s="11" t="s">
+      <c r="Q18" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R18" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S18" s="11">
+      <c r="R18" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S18" s="6">
         <v>20.0</v>
       </c>
-      <c r="T18" s="11" t="s">
+      <c r="T18" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="U18" s="11">
+      <c r="U18" s="6">
         <v>5500.0</v>
       </c>
-      <c r="V18" s="11">
+      <c r="V18" s="6">
         <v>69000.0</v>
       </c>
-      <c r="X18" s="11" t="s">
+      <c r="X18" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="Z18" s="13" t="s">
+      <c r="Z18" s="6" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8">
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="5">
         <v>45576.63496109954</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="B19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="6">
         <v>5.0</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="6">
         <v>2.5</v>
       </c>
-      <c r="P19" s="9" t="s">
+      <c r="P19" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q19" s="9" t="s">
+      <c r="Q19" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R19" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S19" s="9">
+      <c r="R19" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S19" s="6">
         <v>1.0</v>
       </c>
-      <c r="T19" s="9" t="s">
+      <c r="T19" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="U19" s="9">
+      <c r="U19" s="6">
         <v>4300.0</v>
       </c>
-      <c r="V19" s="9">
+      <c r="V19" s="6">
         <v>52000.0</v>
       </c>
-      <c r="X19" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10">
+      <c r="X19" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="5">
         <v>45576.64357231482</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="11" t="s">
+      <c r="B20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="6">
         <v>9.0</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="H20" s="11">
+      <c r="H20" s="6">
         <v>5.0</v>
       </c>
-      <c r="P20" s="11" t="s">
+      <c r="P20" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="Q20" s="11" t="s">
+      <c r="Q20" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R20" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S20" s="11">
+      <c r="R20" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S20" s="6">
         <v>1.0</v>
       </c>
-      <c r="T20" s="11" t="s">
+      <c r="T20" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="U20" s="11">
+      <c r="U20" s="6">
         <v>6500.0</v>
       </c>
-      <c r="V20" s="11">
+      <c r="V20" s="6">
         <v>75000.0</v>
       </c>
-      <c r="X20" s="11" t="s">
+      <c r="X20" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8">
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="5">
         <v>45576.647780011575</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="B21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="6">
         <v>12.0</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="6">
         <v>3.0</v>
       </c>
-      <c r="P21" s="9" t="s">
+      <c r="P21" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="Q21" s="9" t="s">
+      <c r="Q21" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R21" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S21" s="9">
+      <c r="R21" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S21" s="6">
         <v>0.0</v>
       </c>
-      <c r="T21" s="9" t="s">
+      <c r="T21" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="U21" s="9">
+      <c r="U21" s="6">
         <v>12000.0</v>
       </c>
-      <c r="V21" s="9">
+      <c r="V21" s="6">
         <v>147000.0</v>
       </c>
-      <c r="W21" s="9" t="s">
+      <c r="W21" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="X21" s="9" t="s">
+      <c r="X21" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10">
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="5">
         <v>45576.657618321755</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" s="11" t="s">
+      <c r="B22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="6">
         <v>2.0</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="H22" s="11">
+      <c r="H22" s="6">
         <v>50.0</v>
       </c>
-      <c r="P22" s="11" t="s">
+      <c r="P22" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q22" s="11" t="s">
+      <c r="Q22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="R22" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S22" s="11">
+      <c r="R22" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S22" s="6">
         <v>50.0</v>
       </c>
-      <c r="T22" s="11" t="s">
+      <c r="T22" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="U22" s="11">
+      <c r="U22" s="6">
         <v>4800.0</v>
       </c>
-      <c r="V22" s="11">
+      <c r="V22" s="6">
         <v>65000.0</v>
       </c>
-      <c r="W22" s="11" t="s">
+      <c r="W22" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="X22" s="11" t="s">
+      <c r="X22" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="Y22" s="11" t="s">
+      <c r="Y22" s="6" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8">
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="5">
         <v>45576.66412061342</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="B23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="6">
         <v>8.0</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="6">
         <v>15.0</v>
       </c>
-      <c r="O23" s="9" t="s">
+      <c r="O23" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="P23" s="9" t="s">
+      <c r="P23" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q23" s="9" t="s">
+      <c r="Q23" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R23" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S23" s="9">
+      <c r="R23" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S23" s="6">
         <v>85.0</v>
       </c>
-      <c r="T23" s="9" t="s">
+      <c r="T23" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="U23" s="9">
+      <c r="U23" s="6">
         <v>5000.0</v>
       </c>
-      <c r="V23" s="9">
+      <c r="V23" s="6">
         <v>65000.0</v>
       </c>
-      <c r="X23" s="9" t="s">
+      <c r="X23" s="6" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10">
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="5">
         <v>45576.687335462964</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="11" t="s">
+      <c r="B24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="6">
         <v>3.0</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H24" s="11">
+      <c r="H24" s="6">
         <v>6.0</v>
       </c>
-      <c r="P24" s="11" t="s">
+      <c r="P24" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="Q24" s="11" t="s">
+      <c r="Q24" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R24" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S24" s="11">
+      <c r="R24" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S24" s="6">
         <v>20.0</v>
       </c>
-      <c r="T24" s="11" t="s">
+      <c r="T24" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="U24" s="11">
+      <c r="U24" s="6">
         <v>4450.0</v>
       </c>
-      <c r="V24" s="11">
+      <c r="V24" s="6">
         <v>53400.0</v>
       </c>
-      <c r="X24" s="11" t="s">
+      <c r="X24" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="8">
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="5">
         <v>45576.72687866898</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" s="9" t="s">
+      <c r="B25" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="6">
         <v>25.0</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="H25" s="9">
+      <c r="H25" s="6">
         <v>5.0</v>
       </c>
-      <c r="O25" s="9" t="s">
+      <c r="O25" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="P25" s="9" t="s">
+      <c r="P25" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q25" s="9" t="s">
+      <c r="Q25" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R25" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S25" s="9">
+      <c r="R25" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S25" s="6">
         <v>20.0</v>
       </c>
-      <c r="T25" s="9" t="s">
+      <c r="T25" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="U25" s="9">
+      <c r="U25" s="6">
         <v>6400.0</v>
       </c>
-      <c r="V25" s="9">
+      <c r="V25" s="6">
         <v>82000.0</v>
       </c>
-      <c r="X25" s="9" t="s">
+      <c r="X25" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="10">
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="5">
         <v>45576.7496330787</v>
       </c>
-      <c r="B26" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D26" s="11" t="s">
+      <c r="B26" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F26" s="11">
+      <c r="F26" s="6">
         <v>19.0</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="H26" s="11">
+      <c r="H26" s="6">
         <v>5.0</v>
       </c>
-      <c r="O26" s="11" t="s">
+      <c r="O26" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="P26" s="11" t="s">
+      <c r="P26" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q26" s="11" t="s">
+      <c r="Q26" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R26" s="11">
+      <c r="R26" s="6">
         <v>115.0</v>
       </c>
-      <c r="S26" s="11">
+      <c r="S26" s="6">
         <v>20.0</v>
       </c>
-      <c r="T26" s="11" t="s">
+      <c r="T26" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="U26" s="11">
+      <c r="U26" s="6">
         <v>8200.0</v>
       </c>
-      <c r="V26" s="11">
+      <c r="V26" s="6">
         <v>100000.0</v>
       </c>
-      <c r="W26" s="11" t="s">
+      <c r="W26" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="X26" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y26" s="11" t="s">
+      <c r="X26" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y26" s="6" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="8">
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="5">
         <v>45578.624214386575</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="B27" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27" s="6">
         <v>9.0</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="6">
         <v>7.0</v>
       </c>
-      <c r="P27" s="9" t="s">
+      <c r="P27" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="Q27" s="9" t="s">
+      <c r="Q27" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R27" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S27" s="9">
+      <c r="R27" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S27" s="6">
         <v>0.0</v>
       </c>
-      <c r="T27" s="9" t="s">
+      <c r="T27" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="U27" s="9">
+      <c r="U27" s="6">
         <v>4900.0</v>
       </c>
-      <c r="V27" s="9">
+      <c r="V27" s="6">
         <v>61000.0</v>
       </c>
-      <c r="X27" s="9" t="s">
+      <c r="X27" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="10">
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="5">
         <v>45579.53994641204</v>
       </c>
-      <c r="B28" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="11" t="s">
+      <c r="B28" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F28" s="11">
+      <c r="F28" s="6">
         <v>12.0</v>
       </c>
-      <c r="G28" s="11" t="s">
+      <c r="G28" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="O28" s="11" t="s">
+      <c r="O28" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="P28" s="11" t="s">
+      <c r="P28" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q28" s="11" t="s">
+      <c r="Q28" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R28" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S28" s="11">
+      <c r="R28" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S28" s="6">
         <v>50.0</v>
       </c>
-      <c r="T28" s="11" t="s">
+      <c r="T28" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="U28" s="11">
+      <c r="U28" s="6">
         <v>5800.0</v>
       </c>
-      <c r="V28" s="11">
+      <c r="V28" s="6">
         <v>75000.0</v>
       </c>
-      <c r="X28" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8">
+      <c r="X28" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="5">
         <v>45579.62509987269</v>
       </c>
-      <c r="B29" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29" s="9" t="s">
+      <c r="B29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="6">
         <v>9.0</v>
       </c>
-      <c r="G29" s="9" t="s">
+      <c r="G29" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="P29" s="9" t="s">
+      <c r="P29" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q29" s="9" t="s">
+      <c r="Q29" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R29" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S29" s="9">
+      <c r="R29" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S29" s="6">
         <v>0.0</v>
       </c>
-      <c r="T29" s="9" t="s">
+      <c r="T29" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="U29" s="9">
+      <c r="U29" s="6">
         <v>1700.0</v>
       </c>
-      <c r="V29" s="9">
+      <c r="V29" s="6">
         <v>20000.0</v>
       </c>
-      <c r="X29" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10">
+      <c r="X29" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="5">
         <v>45580.67219628472</v>
       </c>
-      <c r="B30" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="11" t="s">
+      <c r="B30" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E30" s="11" t="s">
+      <c r="E30" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="6">
         <v>7.0</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="G30" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="H30" s="11">
+      <c r="H30" s="6">
         <v>1.0</v>
       </c>
-      <c r="O30" s="11" t="s">
+      <c r="O30" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="P30" s="11" t="s">
+      <c r="P30" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q30" s="11" t="s">
+      <c r="Q30" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R30" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S30" s="11">
+      <c r="R30" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S30" s="6">
         <v>99.0</v>
       </c>
-      <c r="T30" s="11" t="s">
+      <c r="T30" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="U30" s="11">
+      <c r="U30" s="6">
         <v>6200.0</v>
       </c>
-      <c r="X30" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8">
+      <c r="X30" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="5">
         <v>45580.673159224534</v>
       </c>
-      <c r="B31" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D31" s="9" t="s">
+      <c r="B31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="F31" s="9">
+      <c r="F31" s="6">
         <v>4.0</v>
       </c>
-      <c r="G31" s="9" t="s">
+      <c r="G31" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31" s="6">
         <v>6.0</v>
       </c>
-      <c r="O31" s="9" t="s">
+      <c r="O31" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="P31" s="9" t="s">
+      <c r="P31" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q31" s="9" t="s">
+      <c r="Q31" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R31" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S31" s="9">
+      <c r="R31" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S31" s="6">
         <v>10.0</v>
       </c>
-      <c r="T31" s="9" t="s">
+      <c r="T31" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="U31" s="9">
+      <c r="U31" s="6">
         <v>4840.0</v>
       </c>
-      <c r="V31" s="9">
+      <c r="V31" s="6">
         <v>58500.0</v>
       </c>
-      <c r="X31" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10">
+      <c r="X31" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="5">
         <v>45580.674445</v>
       </c>
-      <c r="B32" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32" s="11" t="s">
+      <c r="B32" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E32" s="11" t="s">
+      <c r="E32" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="6">
         <v>6.0</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="G32" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="H32" s="11">
+      <c r="H32" s="6">
         <v>8.0</v>
       </c>
-      <c r="O32" s="11" t="s">
+      <c r="O32" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="P32" s="11" t="s">
+      <c r="P32" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q32" s="11" t="s">
+      <c r="Q32" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R32" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S32" s="11">
+      <c r="R32" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S32" s="6">
         <v>0.0</v>
       </c>
-      <c r="T32" s="11" t="s">
+      <c r="T32" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="U32" s="11">
+      <c r="U32" s="6">
         <v>5300.0</v>
       </c>
-      <c r="V32" s="11">
+      <c r="V32" s="6">
         <v>78000.0</v>
       </c>
-      <c r="W32" s="11" t="s">
+      <c r="W32" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="X32" s="11" t="s">
+      <c r="X32" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="8">
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="5">
         <v>45580.68478858796</v>
       </c>
-      <c r="B33" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D33" s="9" t="s">
+      <c r="B33" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F33" s="9">
+      <c r="F33" s="6">
         <v>9.0</v>
       </c>
-      <c r="G33" s="9" t="s">
+      <c r="G33" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="H33" s="9">
+      <c r="H33" s="6">
         <v>3.3</v>
       </c>
-      <c r="O33" s="9" t="s">
+      <c r="O33" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="P33" s="9" t="s">
+      <c r="P33" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q33" s="9" t="s">
+      <c r="Q33" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R33" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S33" s="9">
+      <c r="R33" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S33" s="6">
         <v>20.0</v>
       </c>
-      <c r="T33" s="9" t="s">
+      <c r="T33" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="U33" s="9">
+      <c r="U33" s="6">
         <v>5690.0</v>
       </c>
-      <c r="V33" s="9">
+      <c r="V33" s="6">
         <v>74000.0</v>
       </c>
-      <c r="X33" s="9" t="s">
+      <c r="X33" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="10">
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="5">
         <v>45580.691563726854</v>
       </c>
-      <c r="B34" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D34" s="11" t="s">
+      <c r="B34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D34" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E34" s="11" t="s">
+      <c r="E34" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F34" s="11">
+      <c r="F34" s="6">
         <v>3.0</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="G34" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="H34" s="11">
+      <c r="H34" s="6">
         <v>11.0</v>
       </c>
-      <c r="P34" s="11" t="s">
+      <c r="P34" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q34" s="11" t="s">
+      <c r="Q34" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R34" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S34" s="11">
+      <c r="R34" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S34" s="6">
         <v>40.0</v>
       </c>
-      <c r="T34" s="11" t="s">
+      <c r="T34" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="U34" s="11">
+      <c r="U34" s="6">
         <v>5100.0</v>
       </c>
-      <c r="V34" s="11">
+      <c r="V34" s="6">
         <v>61200.0</v>
       </c>
-      <c r="X34" s="11" t="s">
+      <c r="X34" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8">
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="5">
         <v>45580.70702543981</v>
       </c>
-      <c r="B35" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D35" s="9" t="s">
+      <c r="B35" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F35" s="9">
+      <c r="F35" s="6">
         <v>13.0</v>
       </c>
-      <c r="G35" s="9" t="s">
+      <c r="G35" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="H35" s="9">
+      <c r="H35" s="6">
         <v>3.0</v>
       </c>
-      <c r="P35" s="9" t="s">
+      <c r="P35" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q35" s="9" t="s">
+      <c r="Q35" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R35" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S35" s="9">
+      <c r="R35" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S35" s="6">
         <v>50.0</v>
       </c>
-      <c r="T35" s="9" t="s">
+      <c r="T35" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="9">
+      <c r="U35" s="6">
         <v>5790.0</v>
       </c>
-      <c r="V35" s="9">
+      <c r="V35" s="6">
         <v>72000.0</v>
       </c>
-      <c r="X35" s="9" t="s">
+      <c r="X35" s="6" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="10">
+    <row r="36" ht="22.5" customHeight="1">
+      <c r="A36" s="5">
         <v>45580.719712488426</v>
       </c>
-      <c r="B36" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D36" s="11" t="s">
+      <c r="B36" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E36" s="11" t="s">
+      <c r="E36" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F36" s="11">
+      <c r="F36" s="6">
         <v>14.0</v>
       </c>
-      <c r="G36" s="11" t="s">
+      <c r="G36" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="H36" s="11">
+      <c r="H36" s="6">
         <v>2.5</v>
       </c>
-      <c r="O36" s="11" t="s">
+      <c r="O36" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="P36" s="11" t="s">
+      <c r="P36" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q36" s="11" t="s">
+      <c r="Q36" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R36" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S36" s="11">
+      <c r="R36" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S36" s="6">
         <v>5.0</v>
       </c>
-      <c r="T36" s="11" t="s">
+      <c r="T36" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="U36" s="11">
+      <c r="U36" s="6">
         <v>5700.0</v>
       </c>
-      <c r="V36" s="11">
+      <c r="V36" s="6">
         <v>70000.0</v>
       </c>
-      <c r="W36" s="11" t="s">
+      <c r="W36" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="X36" s="11" t="s">
+      <c r="X36" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="8">
+    <row r="37" ht="22.5" customHeight="1">
+      <c r="A37" s="5">
         <v>45580.80685603009</v>
       </c>
-      <c r="B37" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D37" s="9" t="s">
+      <c r="B37" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F37" s="9">
+      <c r="F37" s="6">
         <v>12.0</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="H37" s="9">
+      <c r="H37" s="6">
         <v>3.75</v>
       </c>
-      <c r="P37" s="9" t="s">
+      <c r="P37" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q37" s="9" t="s">
+      <c r="Q37" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R37" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S37" s="9">
+      <c r="R37" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S37" s="6">
         <v>10.0</v>
       </c>
-      <c r="T37" s="9" t="s">
+      <c r="T37" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="U37" s="9">
+      <c r="U37" s="6">
         <v>6350.0</v>
       </c>
-      <c r="V37" s="9">
+      <c r="V37" s="6">
         <v>750.0</v>
       </c>
-      <c r="X37" s="9" t="s">
+      <c r="X37" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="10">
+    <row r="38" ht="22.5" customHeight="1">
+      <c r="A38" s="5">
         <v>45581.40609495371</v>
       </c>
-      <c r="B38" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C38" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D38" s="11" t="s">
+      <c r="B38" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D38" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E38" s="11" t="s">
+      <c r="E38" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F38" s="11">
+      <c r="F38" s="6">
         <v>7.0</v>
       </c>
-      <c r="G38" s="11" t="s">
+      <c r="G38" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="H38" s="11" t="s">
+      <c r="H38" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="O38" s="11" t="s">
+      <c r="O38" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="P38" s="11" t="s">
+      <c r="P38" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q38" s="11" t="s">
+      <c r="Q38" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R38" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S38" s="11">
+      <c r="R38" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S38" s="6">
         <v>80.0</v>
       </c>
-      <c r="T38" s="11" t="s">
+      <c r="T38" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="U38" s="11">
+      <c r="U38" s="6">
         <v>9000.0</v>
       </c>
-      <c r="V38" s="11">
+      <c r="V38" s="6">
         <v>112000.0</v>
       </c>
-      <c r="W38" s="11" t="s">
+      <c r="W38" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="X38" s="11" t="s">
+      <c r="X38" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8">
+    <row r="39" ht="22.5" customHeight="1">
+      <c r="A39" s="5">
         <v>45581.42516273148</v>
       </c>
-      <c r="B39" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D39" s="9" t="s">
+      <c r="B39" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F39" s="9">
+      <c r="F39" s="6">
         <v>15.0</v>
       </c>
-      <c r="H39" s="9">
+      <c r="H39" s="6">
         <v>2.0</v>
       </c>
-      <c r="P39" s="9" t="s">
+      <c r="P39" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q39" s="9" t="s">
+      <c r="Q39" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R39" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S39" s="9">
+      <c r="R39" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S39" s="6">
         <v>5.0</v>
       </c>
-      <c r="T39" s="9" t="s">
+      <c r="T39" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="U39" s="9">
+      <c r="U39" s="6">
         <v>7150.0</v>
       </c>
-      <c r="V39" s="9">
+      <c r="V39" s="6">
         <v>90000.0</v>
       </c>
-      <c r="W39" s="9" t="s">
+      <c r="W39" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="X39" s="9" t="s">
+      <c r="X39" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="10">
+    <row r="40" ht="22.5" customHeight="1">
+      <c r="A40" s="5">
         <v>45581.42557614583</v>
       </c>
-      <c r="B40" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="11" t="s">
+      <c r="B40" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E40" s="11" t="s">
+      <c r="E40" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="F40" s="11">
+      <c r="F40" s="6">
         <v>10.0</v>
       </c>
-      <c r="G40" s="11" t="s">
+      <c r="G40" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="H40" s="11">
+      <c r="H40" s="6">
         <v>4.2</v>
       </c>
-      <c r="O40" s="11" t="s">
+      <c r="O40" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="P40" s="11" t="s">
+      <c r="P40" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q40" s="11" t="s">
+      <c r="Q40" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R40" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S40" s="11">
+      <c r="R40" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S40" s="6">
         <v>10.0</v>
       </c>
-      <c r="T40" s="11" t="s">
+      <c r="T40" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="U40" s="11">
+      <c r="U40" s="6">
         <v>6600.0</v>
       </c>
-      <c r="V40" s="11">
+      <c r="V40" s="6">
         <v>81000.0</v>
       </c>
-      <c r="X40" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8">
+      <c r="X40" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41" ht="22.5" customHeight="1">
+      <c r="A41" s="5">
         <v>45581.43346863426</v>
       </c>
-      <c r="B41" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D41" s="9" t="s">
+      <c r="B41" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E41" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="6">
         <v>9.0</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G41" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="O41" s="9" t="s">
+      <c r="O41" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="P41" s="9" t="s">
+      <c r="P41" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q41" s="9" t="s">
+      <c r="Q41" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R41" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S41" s="9">
+      <c r="R41" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S41" s="6">
         <v>5.0</v>
       </c>
-      <c r="T41" s="9" t="s">
+      <c r="T41" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="U41" s="9">
+      <c r="U41" s="6">
         <v>5670.0</v>
       </c>
-      <c r="X41" s="9" t="s">
+      <c r="X41" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="10">
+    <row r="42" ht="22.5" customHeight="1">
+      <c r="A42" s="5">
         <v>45581.442221875</v>
       </c>
-      <c r="B42" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D42" s="11" t="s">
+      <c r="B42" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D42" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F42" s="11">
+      <c r="F42" s="6">
         <v>8.0</v>
       </c>
-      <c r="H42" s="11">
+      <c r="H42" s="6">
         <v>10.0</v>
       </c>
-      <c r="P42" s="11" t="s">
+      <c r="P42" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q42" s="11" t="s">
+      <c r="Q42" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R42" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S42" s="11">
+      <c r="R42" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S42" s="6">
         <v>0.0</v>
       </c>
-      <c r="T42" s="11" t="s">
+      <c r="T42" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="U42" s="11">
+      <c r="U42" s="6">
         <v>7400.0</v>
       </c>
-      <c r="V42" s="11">
+      <c r="V42" s="6">
         <v>92500.0</v>
       </c>
-      <c r="X42" s="11" t="s">
+      <c r="X42" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="8">
+    <row r="43" ht="22.5" customHeight="1">
+      <c r="A43" s="5">
         <v>45581.4527799537</v>
       </c>
-      <c r="B43" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D43" s="9" t="s">
+      <c r="B43" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F43" s="9">
+      <c r="F43" s="6">
         <v>10.0</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G43" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="H43" s="9">
+      <c r="H43" s="6">
         <v>3.0</v>
       </c>
-      <c r="P43" s="9" t="s">
+      <c r="P43" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q43" s="9" t="s">
+      <c r="Q43" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R43" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S43" s="9">
+      <c r="R43" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S43" s="6">
         <v>10.0</v>
       </c>
-      <c r="T43" s="9" t="s">
+      <c r="T43" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="U43" s="9">
+      <c r="U43" s="6">
         <v>6900.0</v>
       </c>
-      <c r="W43" s="9" t="s">
+      <c r="W43" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="X43" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="10">
+      <c r="X43" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" ht="22.5" customHeight="1">
+      <c r="A44" s="5">
         <v>45581.57923199074</v>
       </c>
-      <c r="B44" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C44" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D44" s="11" t="s">
+      <c r="B44" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="F44" s="11">
+      <c r="F44" s="6">
         <v>5.0</v>
       </c>
-      <c r="G44" s="11" t="s">
+      <c r="G44" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H44" s="11">
+      <c r="H44" s="6">
         <v>5.0</v>
       </c>
-      <c r="P44" s="11" t="s">
+      <c r="P44" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q44" s="11" t="s">
+      <c r="Q44" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R44" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S44" s="11">
+      <c r="R44" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S44" s="6">
         <v>5.0</v>
       </c>
-      <c r="T44" s="11" t="s">
+      <c r="T44" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="U44" s="11">
+      <c r="U44" s="6">
         <v>5200.0</v>
       </c>
-      <c r="V44" s="11">
+      <c r="V44" s="6">
         <v>67600.0</v>
       </c>
-      <c r="X44" s="11" t="s">
+      <c r="X44" s="6" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="8">
+    <row r="45" ht="22.5" customHeight="1">
+      <c r="A45" s="5">
         <v>45581.96919152778</v>
       </c>
-      <c r="B45" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D45" s="9" t="s">
+      <c r="B45" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D45" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F45" s="9">
+      <c r="F45" s="6">
         <v>19.0</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="H45" s="9">
+      <c r="H45" s="6">
         <v>7.0</v>
       </c>
-      <c r="P45" s="9" t="s">
+      <c r="P45" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q45" s="9" t="s">
+      <c r="Q45" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R45" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S45" s="9">
+      <c r="R45" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S45" s="6">
         <v>5.0</v>
       </c>
-      <c r="T45" s="9" t="s">
+      <c r="T45" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="U45" s="9">
+      <c r="U45" s="6">
         <v>4566.0</v>
       </c>
-      <c r="V45" s="9">
+      <c r="V45" s="6">
         <v>58900.0</v>
       </c>
-      <c r="W45" s="9" t="s">
+      <c r="W45" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="X45" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="10">
+      <c r="X45" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="46" ht="22.5" customHeight="1">
+      <c r="A46" s="5">
         <v>45586.39307476852</v>
       </c>
-      <c r="B46" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C46" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D46" s="11" t="s">
+      <c r="B46" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D46" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="11" t="s">
+      <c r="E46" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="F46" s="11">
+      <c r="F46" s="6">
         <v>10.0</v>
       </c>
-      <c r="G46" s="11" t="s">
+      <c r="G46" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="H46" s="11">
+      <c r="H46" s="6">
         <v>0.0</v>
       </c>
-      <c r="O46" s="11" t="s">
+      <c r="O46" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="P46" s="11" t="s">
+      <c r="P46" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q46" s="11" t="s">
+      <c r="Q46" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R46" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S46" s="11">
+      <c r="R46" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S46" s="6">
         <v>30.0</v>
       </c>
-      <c r="T46" s="11" t="s">
+      <c r="T46" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="U46" s="11">
+      <c r="U46" s="6">
         <v>6300.0</v>
       </c>
-      <c r="V46" s="11">
+      <c r="V46" s="6">
         <v>80000.0</v>
       </c>
-      <c r="W46" s="11" t="s">
+      <c r="W46" s="6" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="8">
+    <row r="47" ht="22.5" customHeight="1">
+      <c r="A47" s="5">
         <v>45587.55625796296</v>
       </c>
-      <c r="B47" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D47" s="9" t="s">
+      <c r="B47" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F47" s="9">
+      <c r="F47" s="6">
         <v>9.0</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="H47" s="9">
+      <c r="H47" s="6">
         <v>-30.0</v>
       </c>
-      <c r="O47" s="9" t="s">
+      <c r="O47" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="P47" s="9" t="s">
+      <c r="P47" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q47" s="9" t="s">
+      <c r="Q47" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R47" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S47" s="9">
+      <c r="R47" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S47" s="6">
         <v>10.0</v>
       </c>
-      <c r="T47" s="9" t="s">
+      <c r="T47" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="U47" s="9">
+      <c r="U47" s="6">
         <v>1890.0</v>
       </c>
-      <c r="V47" s="9">
+      <c r="V47" s="6">
         <v>62680.0</v>
       </c>
-      <c r="W47" s="9" t="s">
+      <c r="W47" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="X47" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z47" s="12" t="s">
+      <c r="X47" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z47" s="6" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="10">
+    <row r="48" ht="22.5" customHeight="1">
+      <c r="A48" s="5">
         <v>45588.49461217593</v>
       </c>
-      <c r="B48" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C48" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D48" s="11" t="s">
+      <c r="B48" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E48" s="11" t="s">
+      <c r="E48" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F48" s="11">
+      <c r="F48" s="6">
         <v>2.0</v>
       </c>
-      <c r="G48" s="11" t="s">
+      <c r="G48" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="H48" s="11">
+      <c r="H48" s="6">
         <v>10.0</v>
       </c>
-      <c r="P48" s="11" t="s">
+      <c r="P48" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="Q48" s="11" t="s">
+      <c r="Q48" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R48" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S48" s="11">
+      <c r="R48" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S48" s="6">
         <v>0.0</v>
       </c>
-      <c r="T48" s="11" t="s">
+      <c r="T48" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="U48" s="11">
+      <c r="U48" s="6">
         <v>3900.0</v>
       </c>
-      <c r="V48" s="11">
+      <c r="V48" s="6">
         <v>47200.0</v>
       </c>
-      <c r="X48" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8">
+      <c r="X48" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="49" ht="22.5" customHeight="1">
+      <c r="A49" s="5">
         <v>45588.49979001157</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B49" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D49" s="9" t="s">
+      <c r="C49" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E49" s="9" t="s">
+      <c r="E49" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F49" s="9">
+      <c r="F49" s="6">
         <v>14.0</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G49" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="H49" s="9">
+      <c r="H49" s="6">
         <v>0.0</v>
       </c>
-      <c r="I49" s="9">
+      <c r="I49" s="6">
         <v>7.0</v>
       </c>
-      <c r="J49" s="9" t="s">
+      <c r="J49" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="K49" s="9">
+      <c r="K49" s="6">
         <v>95.0</v>
       </c>
-      <c r="L49" s="9">
+      <c r="L49" s="6">
         <v>110000.0</v>
       </c>
-      <c r="M49" s="9" t="s">
+      <c r="M49" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="N49" s="9" t="s">
+      <c r="N49" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="10">
+    <row r="50" ht="22.5" customHeight="1">
+      <c r="A50" s="5">
         <v>45588.49981325232</v>
       </c>
-      <c r="B50" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C50" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D50" s="11" t="s">
+      <c r="B50" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E50" s="11" t="s">
+      <c r="E50" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F50" s="11">
+      <c r="F50" s="6">
         <v>7.0</v>
       </c>
-      <c r="G50" s="11" t="s">
+      <c r="G50" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="H50" s="11">
+      <c r="H50" s="6">
         <v>0.0</v>
       </c>
-      <c r="P50" s="11" t="s">
+      <c r="P50" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="Q50" s="11" t="s">
+      <c r="Q50" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R50" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S50" s="11">
+      <c r="R50" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S50" s="6">
         <v>90.0</v>
       </c>
-      <c r="T50" s="11" t="s">
+      <c r="T50" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="U50" s="11">
+      <c r="U50" s="6">
         <v>5800.0</v>
       </c>
-      <c r="V50" s="11">
+      <c r="V50" s="6">
         <v>70000.0</v>
       </c>
-      <c r="W50" s="11" t="s">
+      <c r="W50" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="X50" s="11" t="s">
+      <c r="X50" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="8">
+    <row r="51" ht="22.5" customHeight="1">
+      <c r="A51" s="5">
         <v>45588.573026666665</v>
       </c>
-      <c r="B51" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D51" s="9" t="s">
+      <c r="B51" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E51" s="9" t="s">
+      <c r="E51" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F51" s="9">
+      <c r="F51" s="6">
         <v>3.0</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="H51" s="9">
+      <c r="H51" s="6">
         <v>5.0</v>
       </c>
-      <c r="P51" s="9" t="s">
+      <c r="P51" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="Q51" s="9" t="s">
+      <c r="Q51" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R51" s="9">
-        <v>100.0</v>
-      </c>
-      <c r="S51" s="9">
+      <c r="R51" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S51" s="6">
         <v>90.0</v>
       </c>
-      <c r="T51" s="9" t="s">
+      <c r="T51" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="U51" s="9">
+      <c r="U51" s="6">
         <v>4670.0</v>
       </c>
-      <c r="V51" s="9">
+      <c r="V51" s="6">
         <v>55000.0</v>
       </c>
-      <c r="W51" s="9" t="s">
+      <c r="W51" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="X51" s="9" t="s">
+      <c r="X51" s="6" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="10">
+    <row r="52" ht="22.5" customHeight="1">
+      <c r="A52" s="5">
         <v>45588.633891562495</v>
       </c>
-      <c r="B52" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C52" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D52" s="11" t="s">
+      <c r="B52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E52" s="11" t="s">
+      <c r="E52" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F52" s="11">
+      <c r="F52" s="6">
         <v>3.0</v>
       </c>
-      <c r="G52" s="11" t="s">
+      <c r="G52" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="H52" s="11">
+      <c r="H52" s="6">
         <v>5.0</v>
       </c>
-      <c r="O52" s="11" t="s">
+      <c r="O52" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="P52" s="11" t="s">
+      <c r="P52" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="Q52" s="11" t="s">
+      <c r="Q52" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R52" s="11">
-        <v>100.0</v>
-      </c>
-      <c r="S52" s="11">
+      <c r="R52" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S52" s="6">
         <v>90.0</v>
       </c>
-      <c r="T52" s="11" t="s">
+      <c r="T52" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="U52" s="11">
+      <c r="U52" s="6">
         <v>4700.0</v>
       </c>
-      <c r="V52" s="11">
+      <c r="V52" s="6">
         <v>58000.0</v>
       </c>
-      <c r="W52" s="11" t="s">
+      <c r="W52" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="X52" s="11" t="s">
+      <c r="X52" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="15">
+    <row r="53" ht="22.5" customHeight="1">
+      <c r="A53" s="5">
         <v>45590.73276068287</v>
       </c>
-      <c r="B53" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="C53" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D53" s="16" t="s">
+      <c r="B53" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D53" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E53" s="16" t="s">
+      <c r="E53" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="F53" s="16">
+      <c r="F53" s="6">
         <v>4.5</v>
       </c>
-      <c r="G53" s="16" t="s">
+      <c r="G53" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="H53" s="16">
+      <c r="H53" s="6">
         <v>0.0</v>
       </c>
-      <c r="O53" s="16" t="s">
+      <c r="O53" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="P53" s="16" t="s">
+      <c r="P53" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q53" s="16" t="s">
+      <c r="Q53" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R53" s="16">
-        <v>100.0</v>
-      </c>
-      <c r="S53" s="16">
+      <c r="R53" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="S53" s="6">
         <v>0.0</v>
       </c>
-      <c r="T53" s="16" t="s">
+      <c r="T53" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="U53" s="16">
+      <c r="U53" s="6">
         <v>3700.0</v>
       </c>
-      <c r="X53" s="16" t="s">
+      <c r="X53" s="6" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>